<commit_message>
Regenerate all figures at 300 dpi on corrected-data baseline
- Set savefig dpi 150->300 across 8 figure notebooks (includes Demand,
  PV vs Demand, Weather data, DT Architecture previously missed)
- Re-execute under eden_phd env against corrected data_prep inputs
  (real demand, fixed cost units); all 7 manuscript figures now 300 dpi
- Regenerate scenario/sensitivity/full-year KPI tables from corrected model
</commit_message>
<xml_diff>
--- a/EdenCampus_PhD/04_results/tables/full_year_scenario_comparison.xlsx
+++ b/EdenCampus_PhD/04_results/tables/full_year_scenario_comparison.xlsx
@@ -520,7 +520,7 @@
         <v>381.4</v>
       </c>
       <c r="L2" t="n">
-        <v>458324.8</v>
+        <v>539</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         <v>2400.9</v>
       </c>
       <c r="D3" t="n">
-        <v>1485.6</v>
+        <v>1495.6</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -548,19 +548,19 @@
         <v>38.8</v>
       </c>
       <c r="H3" t="n">
-        <v>38.1</v>
+        <v>37.7</v>
       </c>
       <c r="I3" t="n">
-        <v>1.4</v>
+        <v>39.7</v>
       </c>
       <c r="J3" t="n">
         <v>217.2</v>
       </c>
       <c r="K3" t="n">
-        <v>346.1</v>
+        <v>348.5</v>
       </c>
       <c r="L3" t="n">
-        <v>415959.2</v>
+        <v>468</v>
       </c>
     </row>
     <row r="4">
@@ -576,7 +576,7 @@
         <v>2400.9</v>
       </c>
       <c r="D4" t="n">
-        <v>2142.6</v>
+        <v>2122.2</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -588,19 +588,19 @@
         <v>35</v>
       </c>
       <c r="H4" t="n">
-        <v>10.8</v>
+        <v>11.6</v>
       </c>
       <c r="I4" t="n">
-        <v>-32.1</v>
+        <v>1.4</v>
       </c>
       <c r="J4" t="n">
         <v>195.7</v>
       </c>
       <c r="K4" t="n">
-        <v>499.2</v>
+        <v>494.5</v>
       </c>
       <c r="L4" t="n">
-        <v>600230.1</v>
+        <v>683.3</v>
       </c>
     </row>
     <row r="5">
@@ -616,7 +616,7 @@
         <v>2400.9</v>
       </c>
       <c r="D5" t="n">
-        <v>1573.2</v>
+        <v>1573.3</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -631,7 +631,7 @@
         <v>34.5</v>
       </c>
       <c r="I5" t="n">
-        <v>1.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J5" t="n">
         <v>220.5</v>
@@ -640,7 +640,7 @@
         <v>366.6</v>
       </c>
       <c r="L5" t="n">
-        <v>440927.2</v>
+        <v>515.6</v>
       </c>
     </row>
     <row r="6">
@@ -656,7 +656,7 @@
         <v>2400.9</v>
       </c>
       <c r="D6" t="n">
-        <v>2013.6</v>
+        <v>1820.1</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -668,19 +668,19 @@
         <v>42.7</v>
       </c>
       <c r="H6" t="n">
-        <v>16.1</v>
+        <v>24.2</v>
       </c>
       <c r="I6" t="n">
-        <v>-32.1</v>
+        <v>40</v>
       </c>
       <c r="J6" t="n">
         <v>238.8</v>
       </c>
       <c r="K6" t="n">
-        <v>469.2</v>
+        <v>424.1</v>
       </c>
       <c r="L6" t="n">
-        <v>564249.6</v>
+        <v>628.4</v>
       </c>
     </row>
   </sheetData>
@@ -947,7 +947,7 @@
         <v>20.103715976</v>
       </c>
       <c r="C2" t="n">
-        <v>226.2283567839306</v>
+        <v>229.2078497041942</v>
       </c>
       <c r="D2" t="n">
         <v>246.3242676246747</v>
@@ -963,7 +963,7 @@
         <v>31.986103672</v>
       </c>
       <c r="C3" t="n">
-        <v>182.8457653896541</v>
+        <v>184.0843704359021</v>
       </c>
       <c r="D3" t="n">
         <v>214.7800372266234</v>
@@ -979,7 +979,7 @@
         <v>81.14646642732561</v>
       </c>
       <c r="C4" t="n">
-        <v>134.5343093874333</v>
+        <v>134.5446151938731</v>
       </c>
       <c r="D4" t="n">
         <v>214.7302353741933</v>
@@ -995,7 +995,7 @@
         <v>112.1335606491616</v>
       </c>
       <c r="C5" t="n">
-        <v>66.73804216379365</v>
+        <v>66.73804216379364</v>
       </c>
       <c r="D5" t="n">
         <v>176.3914901131404</v>
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>143.7658265478713</v>
+        <v>143.7658064879308</v>
       </c>
       <c r="C6" t="n">
         <v>44.69697094927113</v>
@@ -1024,10 +1024,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>131.539176457538</v>
+        <v>131.5391903258646</v>
       </c>
       <c r="C7" t="n">
-        <v>39.91203696809012</v>
+        <v>39.91208257876501</v>
       </c>
       <c r="D7" t="n">
         <v>168.3248471554659</v>
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>128.0862454802077</v>
+        <v>128.0861929281086</v>
       </c>
       <c r="C8" t="n">
         <v>40.56214315288391</v>
@@ -1075,7 +1075,7 @@
         <v>84.26197973703319</v>
       </c>
       <c r="C10" t="n">
-        <v>98.72553937643559</v>
+        <v>98.88125530092397</v>
       </c>
       <c r="D10" t="n">
         <v>181.759449816913</v>
@@ -1091,7 +1091,7 @@
         <v>43.8955037612</v>
       </c>
       <c r="C11" t="n">
-        <v>164.8684624987261</v>
+        <v>164.9630056361315</v>
       </c>
       <c r="D11" t="n">
         <v>208.333666946658</v>
@@ -1107,7 +1107,7 @@
         <v>19.8103889632</v>
       </c>
       <c r="C12" t="n">
-        <v>204.6234767264434</v>
+        <v>206.8064057234156</v>
       </c>
       <c r="D12" t="n">
         <v>224.3770958568271</v>
@@ -1123,7 +1123,7 @@
         <v>9.745780574799999</v>
       </c>
       <c r="C13" t="n">
-        <v>229.3887877941529</v>
+        <v>232.7593535225859</v>
       </c>
       <c r="D13" t="n">
         <v>239.1345683689529</v>
@@ -1170,7 +1170,7 @@
         <v>20.103715976</v>
       </c>
       <c r="C2" t="n">
-        <v>322.6191069513143</v>
+        <v>313.6103112617952</v>
       </c>
       <c r="D2" t="n">
         <v>246.3242676246747</v>
@@ -1183,10 +1183,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>31.95106005155624</v>
+        <v>31.95084207340327</v>
       </c>
       <c r="C3" t="n">
-        <v>260.4396823362515</v>
+        <v>260.3637187178642</v>
       </c>
       <c r="D3" t="n">
         <v>214.7800372266234</v>
@@ -1199,10 +1199,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>77.56628642971914</v>
+        <v>77.5657877228209</v>
       </c>
       <c r="C4" t="n">
-        <v>209.3842613138389</v>
+        <v>209.2387653335879</v>
       </c>
       <c r="D4" t="n">
         <v>214.7302353741933</v>
@@ -1215,10 +1215,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>104.1316727145487</v>
+        <v>104.1251964353914</v>
       </c>
       <c r="C5" t="n">
-        <v>113.0591516826708</v>
+        <v>112.9927154226331</v>
       </c>
       <c r="D5" t="n">
         <v>176.3914901131404</v>
@@ -1231,10 +1231,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>126.692971142366</v>
+        <v>126.7379350421787</v>
       </c>
       <c r="C6" t="n">
-        <v>81.71762676955164</v>
+        <v>81.66722587840393</v>
       </c>
       <c r="D6" t="n">
         <v>185.4448065895326</v>
@@ -1247,10 +1247,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>109.1715487487218</v>
+        <v>109.155196032132</v>
       </c>
       <c r="C7" t="n">
-        <v>70.46600594950974</v>
+        <v>70.45932338492976</v>
       </c>
       <c r="D7" t="n">
         <v>168.3248471554659</v>
@@ -1263,10 +1263,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>110.0235311419779</v>
+        <v>110.0312271993092</v>
       </c>
       <c r="C8" t="n">
-        <v>67.13649037284802</v>
+        <v>67.11778947659522</v>
       </c>
       <c r="D8" t="n">
         <v>165.8237946892123</v>
@@ -1279,10 +1279,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>110.0865936846299</v>
+        <v>110.0846358601175</v>
       </c>
       <c r="C9" t="n">
-        <v>77.47144164996216</v>
+        <v>77.45582305808107</v>
       </c>
       <c r="D9" t="n">
         <v>175.455120184745</v>
@@ -1295,10 +1295,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>78.75869274185867</v>
+        <v>78.76112347893786</v>
       </c>
       <c r="C10" t="n">
-        <v>129.0286588236774</v>
+        <v>129.0220584543905</v>
       </c>
       <c r="D10" t="n">
         <v>181.759449816913</v>
@@ -1311,10 +1311,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>41.93314610514992</v>
+        <v>41.94117520105057</v>
       </c>
       <c r="C11" t="n">
-        <v>214.7000766421246</v>
+        <v>214.8183571912408</v>
       </c>
       <c r="D11" t="n">
         <v>208.333666946658</v>
@@ -1327,10 +1327,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>19.79105718943641</v>
+        <v>19.79157605244875</v>
       </c>
       <c r="C12" t="n">
-        <v>278.9577385648402</v>
+        <v>278.8975384319139</v>
       </c>
       <c r="D12" t="n">
         <v>224.3770958568271</v>
@@ -1346,7 +1346,7 @@
         <v>9.745780574799999</v>
       </c>
       <c r="C13" t="n">
-        <v>317.660051600424</v>
+        <v>306.5727740540944</v>
       </c>
       <c r="D13" t="n">
         <v>239.1345683689529</v>
@@ -1393,7 +1393,7 @@
         <v>20.103715976</v>
       </c>
       <c r="C2" t="n">
-        <v>226.2724382161883</v>
+        <v>226.0965003338534</v>
       </c>
       <c r="D2" t="n">
         <v>246.3242676246747</v>
@@ -1537,7 +1537,7 @@
         <v>43.42138219462257</v>
       </c>
       <c r="C11" t="n">
-        <v>167.4197481113175</v>
+        <v>168.0200695836507</v>
       </c>
       <c r="D11" t="n">
         <v>208.333666946658</v>
@@ -1553,7 +1553,7 @@
         <v>19.8103889632</v>
       </c>
       <c r="C12" t="n">
-        <v>204.9431715852854</v>
+        <v>205.1458017412619</v>
       </c>
       <c r="D12" t="n">
         <v>224.3770958568271</v>
@@ -1569,7 +1569,7 @@
         <v>9.745780574799999</v>
       </c>
       <c r="C13" t="n">
-        <v>229.3887877941529</v>
+        <v>228.8646519595089</v>
       </c>
       <c r="D13" t="n">
         <v>239.1345683689529</v>
@@ -1616,7 +1616,7 @@
         <v>20.103715976</v>
       </c>
       <c r="C2" t="n">
-        <v>322.6191069513143</v>
+        <v>256.995886981395</v>
       </c>
       <c r="D2" t="n">
         <v>246.3242676246747</v>
@@ -1632,7 +1632,7 @@
         <v>31.986103672</v>
       </c>
       <c r="C3" t="n">
-        <v>260.4025344631719</v>
+        <v>227.3830063993495</v>
       </c>
       <c r="D3" t="n">
         <v>214.7800372266234</v>
@@ -1648,7 +1648,7 @@
         <v>81.194437278</v>
       </c>
       <c r="C4" t="n">
-        <v>206.0171900178635</v>
+        <v>206.62387106047</v>
       </c>
       <c r="D4" t="n">
         <v>214.7302353741933</v>
@@ -1664,7 +1664,7 @@
         <v>118.9784377972</v>
       </c>
       <c r="C5" t="n">
-        <v>101.2222322828613</v>
+        <v>101.1484265985943</v>
       </c>
       <c r="D5" t="n">
         <v>176.3914901131404</v>
@@ -1680,7 +1680,7 @@
         <v>157.0100742604</v>
       </c>
       <c r="C6" t="n">
-        <v>59.98417335240736</v>
+        <v>59.9726121381609</v>
       </c>
       <c r="D6" t="n">
         <v>185.4448065895326</v>
@@ -1693,10 +1693,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>157.9180141290699</v>
+        <v>157.9141139080972</v>
       </c>
       <c r="C7" t="n">
-        <v>36.91249018247384</v>
+        <v>36.90252012911148</v>
       </c>
       <c r="D7" t="n">
         <v>168.3248471554659</v>
@@ -1709,10 +1709,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>157.1020186193177</v>
+        <v>157.1096922795564</v>
       </c>
       <c r="C8" t="n">
-        <v>38.50198972260022</v>
+        <v>38.48329024654194</v>
       </c>
       <c r="D8" t="n">
         <v>165.8237946892123</v>
@@ -1728,7 +1728,7 @@
         <v>137.4382846624</v>
       </c>
       <c r="C9" t="n">
-        <v>57.24999146573936</v>
+        <v>58.67116665836402</v>
       </c>
       <c r="D9" t="n">
         <v>175.455120184745</v>
@@ -1744,7 +1744,7 @@
         <v>89.52794195199999</v>
       </c>
       <c r="C10" t="n">
-        <v>121.1521525108686</v>
+        <v>123.4647315644024</v>
       </c>
       <c r="D10" t="n">
         <v>181.759449816913</v>
@@ -1760,7 +1760,7 @@
         <v>43.8955037612</v>
       </c>
       <c r="C11" t="n">
-        <v>212.9076526759463</v>
+        <v>214.413685064625</v>
       </c>
       <c r="D11" t="n">
         <v>208.333666946658</v>
@@ -1776,7 +1776,7 @@
         <v>19.8103889632</v>
       </c>
       <c r="C12" t="n">
-        <v>278.9342206158119</v>
+        <v>244.8023298589628</v>
       </c>
       <c r="D12" t="n">
         <v>224.3770958568271</v>
@@ -1792,7 +1792,7 @@
         <v>9.745780574799999</v>
       </c>
       <c r="C13" t="n">
-        <v>317.660051600424</v>
+        <v>251.2495688251057</v>
       </c>
       <c r="D13" t="n">
         <v>239.1345683689529</v>

</xml_diff>